<commit_message>
feat: passeio externo, interno ou ambos no vídeo; nomes dos arquivos com AAAAMMDD-HHMM
- opção Passeio (aba Vídeo da planilha e passo Conferir): volta baixa por fora,
  por dentro a 1,0 m/s desde 3,5 m antes da porta (fov 75°), ou ambos com corte;
  interior só quando o voo acha a porta de entrada
- câmeras das tomadas começam pela isométrica e perdem a lateral
- Entardecer com céu mais limpo e sem aquecimento duplo; filtro degradê no céu
- todas as exportações levam carimbo AAAAMMDD-HHMM na hora local
- ADR-32 e README

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/modelos/obra-dani.xlsx
+++ b/public/modelos/obra-dani.xlsx
@@ -640,7 +640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -714,6 +714,11 @@
           <t>fps</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>passeio</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -786,6 +791,11 @@
           <t>30</t>
         </is>
       </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>externo</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -858,6 +868,11 @@
           <t>24</t>
         </is>
       </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>interno</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -898,6 +913,11 @@
       <c r="K4" t="inlineStr">
         <is>
           <t>Fade-in</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>ambos</t>
         </is>
       </c>
     </row>
@@ -5740,7 +5760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5889,8 +5909,25 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Passeio</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>externo</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Fim do vídeo: volta por fora, por dentro (entra pela porta) ou ambos. Interno pede casa com porta de entrada.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <dataValidations count="7">
+  <dataValidations count="8">
     <dataValidation sqref="B2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
       <formula1>Listas!$H$2:$H$4</formula1>
     </dataValidation>
@@ -5911,6 +5948,9 @@
     </dataValidation>
     <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
       <formula1>Listas!$M$2:$M$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
+      <formula1>Listas!$O$2:$O$4</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: sequência do vídeo com narração, fotos emolduradas e trilhas sonoras
- cartões: Planilha, Projeto IFC, Apresentação (vídeos e áudios de
  narração), Fotos e o novo Trilha sonora
- Conferir: painel "Sequência do vídeo" para ordenar vídeos, narrações e
  fotos (↑ ↓ ou arrastar), duração das fotos e entrada e volume de cada
  trilha (início, antes de um item, final)
- fotos entram emolduradas (passe-partout, filete dourado, sombra, legenda
  com data, etapa e descrição, zoom lento) sobre a obra no dia delas
- mixagem: trilhas em laço com cruzamentos, ducking sob a voz, fade-out
  final e último 0,3 s em silêncio; respiro de 1 s antes da marca
- planilha: abas Sequência e Trilhas (ler, escrever e modelo)
- ADR-34 e README

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/modelos/obra-dani.xlsx
+++ b/public/modelos/obra-dani.xlsx
@@ -14,9 +14,11 @@
     <sheet name="Vínculos" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Falas" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Fotos" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Vídeo" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Documento" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Listas" sheetId="10" state="hidden" r:id="rId10"/>
+    <sheet name="Sequência" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Trilhas" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Vídeo" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Documento" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Listas" sheetId="12" state="hidden" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -493,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B22"/>
+  <dimension ref="B2:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -534,7 +536,7 @@
     <row r="8">
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2. No app, passo Carregar: envie esta planilha e, em cartões separados, o IFC (opcional), os vídeos das falas e as fotos.</t>
+          <t>2. No app, passo Carregar: envie esta planilha e, em cartões separados, o IFC (opcional), a apresentação (vídeos e áudios de narração), as fotos e as trilhas sonoras.</t>
         </is>
       </c>
     </row>
@@ -600,29 +602,43 @@
     <row r="18">
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Vídeo: formato, duração, qualidade e luz do vídeo.</t>
+          <t>Sequência: opcional. A ordem do vídeo (fala, narração, foto); vazia = falas na ordem e fotos pela data. Também se ajusta no passo Conferir.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Documento: título, destinatário, observações e seções do PDF/DOCX.</t>
+          <t>Trilhas: opcional. Onde cada música entra (início, final ou "antes de &lt;arquivo&gt;") e o volume (0 a 100).</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="3" t="inlineStr"/>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Vídeo: formato, duração, qualidade e luz do vídeo.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="B21" s="3" t="inlineStr">
         <is>
+          <t>Documento: título, destinatário, observações e seções do PDF/DOCX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="3" t="inlineStr">
+        <is>
           <t>Os campos com seta têm lista de valores. Não renomeie as abas nem os cabeçalhos.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="3" t="inlineStr">
+    <row r="24">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Manual completo: https://marceloclr.github.io/dani/manual.html</t>
         </is>
@@ -640,7 +656,381 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>campo</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>observação</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Formato</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>vertical 9:16</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>Vertical para Reels e Stories; horizontal para YouTube e apresentações.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Duração (s)</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Vazio = soma das falas e narrações, mais as fotos (ou 30 s sem nada). Sem voz, mas com fotos ou trilhas: o tempo da obra. Máximo 120 s.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Quadros por segundo</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Qualidade</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>máxima</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Máxima renderiza com mais definição e demora mais.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Aparência</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Realista</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Luz</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Dia</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Ciclo = o dia corre do amanhecer à noite durante o voo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Animação</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Progressivo</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Como cada elemento surge durante a sua etapa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Marca no canto</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Faixa com o monograma, o nome e o slogan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Passeio</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>externo</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Fim do vídeo: volta por fora, por dentro (entra pela porta) ou ambos. Interno pede casa com porta de entrada.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="8">
+    <dataValidation sqref="B2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
+      <formula1>Listas!$H$2:$H$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
+      <formula1>Listas!$N$2:$N$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
+      <formula1>Listas!$I$2:$I$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="B6" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
+      <formula1>Listas!$L$2:$L$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="B7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
+      <formula1>Listas!$J$2:$J$6</formula1>
+    </dataValidation>
+    <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
+      <formula1>Listas!$K$2:$K$6</formula1>
+    </dataValidation>
+    <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
+      <formula1>Listas!$M$2:$M$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
+      <formula1>Listas!$O$2:$O$4</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002C2C2C"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>campo</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>observação</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Título</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Relatório de acompanhamento da obra</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Destinatário</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Família Exemplo</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Observações</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Texto livre no fim do documento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Ficha da obra</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Etapas</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Tabela do cronograma, avanço e desvios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Linha do tempo em imagens</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Quadros do vídeo gerado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Fotos da obra</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Referência ao vídeo</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Nome, duração e código de conferência do MP4.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="5">
+    <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
+      <formula1>Listas!$M$2:$M$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="B6" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
+      <formula1>Listas!$M$2:$M$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="B7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
+      <formula1>Listas!$M$2:$M$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
+      <formula1>Listas!$M$2:$M$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
+      <formula1>Listas!$M$2:$M$3</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002C2C2C"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -719,6 +1109,16 @@
           <t>passeio</t>
         </is>
       </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>tiposeq</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>entra</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -796,6 +1196,16 @@
           <t>externo</t>
         </is>
       </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>fala</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>início</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -873,6 +1283,16 @@
           <t>interno</t>
         </is>
       </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>narração</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>final</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -918,6 +1338,11 @@
       <c r="O4" t="inlineStr">
         <is>
           <t>ambos</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>foto</t>
         </is>
       </c>
     </row>
@@ -5760,197 +6185,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>campo</t>
+          <t>ordem</t>
         </is>
       </c>
       <c r="B1" s="5" t="inlineStr">
         <is>
-          <t>valor</t>
+          <t>tipo</t>
         </is>
       </c>
       <c r="C1" s="5" t="inlineStr">
         <is>
-          <t>observação</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>Formato</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>vertical 9:16</t>
-        </is>
-      </c>
-      <c r="C2" s="8" t="inlineStr">
-        <is>
-          <t>Vertical para Reels e Stories; horizontal para YouTube e apresentações.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>Duração (s)</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr"/>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>Vazio = soma das falas (ou 30 s sem falas). Máximo 120 s.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Quadros por segundo</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Qualidade</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>máxima</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>Máxima renderiza com mais definição e demora mais.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Aparência</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>Realista</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Luz</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Dia</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>Ciclo = o dia corre do amanhecer à noite durante o voo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>Animação</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Progressivo</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>Como cada elemento surge durante a sua etapa.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Marca no canto</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Faixa com o monograma, o nome e o slogan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Passeio</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>externo</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>Fim do vídeo: volta por fora, por dentro (entra pela porta) ou ambos. Interno pede casa com porta de entrada.</t>
+          <t>arquivo</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>duracao_s</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="8">
-    <dataValidation sqref="B2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
-      <formula1>Listas!$H$2:$H$4</formula1>
-    </dataValidation>
-    <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
-      <formula1>Listas!$N$2:$N$3</formula1>
-    </dataValidation>
-    <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
-      <formula1>Listas!$I$2:$I$3</formula1>
-    </dataValidation>
-    <dataValidation sqref="B6" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
-      <formula1>Listas!$L$2:$L$3</formula1>
-    </dataValidation>
-    <dataValidation sqref="B7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
-      <formula1>Listas!$J$2:$J$6</formula1>
-    </dataValidation>
-    <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
-      <formula1>Listas!$K$2:$K$6</formula1>
-    </dataValidation>
-    <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
-      <formula1>Listas!$M$2:$M$3</formula1>
-    </dataValidation>
-    <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
-      <formula1>Listas!$O$2:$O$4</formula1>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B400" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
+      <formula1>Listas!$P$2:$P$4</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5964,163 +6233,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>campo</t>
+          <t>arquivo</t>
         </is>
       </c>
       <c r="B1" s="5" t="inlineStr">
         <is>
-          <t>valor</t>
+          <t>entra</t>
         </is>
       </c>
       <c r="C1" s="5" t="inlineStr">
         <is>
-          <t>observação</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>Título</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>Relatório de acompanhamento da obra</t>
-        </is>
-      </c>
-      <c r="C2" s="8" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>Destinatário</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>Família Exemplo</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Observações</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr"/>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>Texto livre no fim do documento.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Ficha da obra</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Etapas</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>Tabela do cronograma, avanço e desvios.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Linha do tempo em imagens</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>Quadros do vídeo gerado.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>Fotos da obra</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Referência ao vídeo</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Nome, duração e código de conferência do MP4.</t>
+          <t>volume</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="5">
-    <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
-      <formula1>Listas!$M$2:$M$3</formula1>
-    </dataValidation>
-    <dataValidation sqref="B6" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
-      <formula1>Listas!$M$2:$M$3</formula1>
-    </dataValidation>
-    <dataValidation sqref="B7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
-      <formula1>Listas!$M$2:$M$3</formula1>
-    </dataValidation>
-    <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
-      <formula1>Listas!$M$2:$M$3</formula1>
-    </dataValidation>
-    <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
-      <formula1>Listas!$M$2:$M$3</formula1>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
+      <formula1>Listas!$Q$2:$Q$3</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>